<commit_message>
dloc -> changed lines
</commit_message>
<xml_diff>
--- a/Data/Glados/glados.xlsx
+++ b/Data/Glados/glados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\makinoyuuki\Desktop\ESEM2026\Data\Glados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19D20B10-16BB-4FD9-A9F8-D4D28569BDDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A532F3D-2E51-41AE-A682-77B01566881F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{76F834DE-5EFC-4D6B-9741-493A547AC4EA}"/>
   </bookViews>
@@ -187,10 +187,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>dloc</t>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t xml:space="preserve">lines_added </t>
     <phoneticPr fontId="1"/>
   </si>
@@ -386,6 +382,10 @@
   </si>
   <si>
     <t>-</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>changed_lines</t>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -536,7 +536,7 @@
     <tableColumn id="1" xr3:uid="{5C7DFBEE-0D79-4A94-BFD4-E8F1FB47AC2F}" name="test_name" dataDxfId="2"/>
     <tableColumn id="2" xr3:uid="{30D127E9-6770-460C-AFEA-9A821352C371}" name="effort" dataDxfId="1"/>
     <tableColumn id="3" xr3:uid="{115F9ED8-8869-42CD-9282-82B281C22540}" name="sequence_number"/>
-    <tableColumn id="4" xr3:uid="{BD43728E-7EA1-464D-8FEF-4DBB03D04C8A}" name="dloc">
+    <tableColumn id="4" xr3:uid="{BD43728E-7EA1-464D-8FEF-4DBB03D04C8A}" name="changed_lines">
       <calculatedColumnFormula>E2+F2</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="5" xr3:uid="{A4005904-B5AE-4A4D-A2FE-AE78D8BCE01E}" name="lines_added "/>
@@ -919,16 +919,16 @@
         <v>33</v>
       </c>
       <c r="D1" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="E1" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>39</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>40</v>
       </c>
       <c r="H1" s="4" t="s">
         <v>34</v>
@@ -940,37 +940,37 @@
         <v>36</v>
       </c>
       <c r="K1" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="L1" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="M1" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="L1" s="4" t="s">
-        <v>50</v>
-      </c>
-      <c r="M1" s="4" t="s">
+      <c r="N1" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="O1" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="O1" s="4" t="s">
+      <c r="P1" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="P1" s="4" t="s">
+      <c r="Q1" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="Q1" s="4" t="s">
+      <c r="R1" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="R1" s="4" t="s">
+      <c r="S1" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="S1" s="4" t="s">
+      <c r="T1" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="T1" s="4" t="s">
-        <v>49</v>
-      </c>
       <c r="U1" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -978,7 +978,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C2" t="s">
         <v>1</v>
@@ -994,7 +994,7 @@
         <v>60</v>
       </c>
       <c r="G2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H2">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -1007,13 +1007,13 @@
         <v>4</v>
       </c>
       <c r="K2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="L2">
         <v>0</v>
       </c>
       <c r="U2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -1021,7 +1021,7 @@
         <v>0</v>
       </c>
       <c r="B3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C3" t="s">
         <v>1</v>
@@ -1037,7 +1037,7 @@
         <v>60</v>
       </c>
       <c r="G3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H3">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -1050,13 +1050,13 @@
         <v>2415.90552710055</v>
       </c>
       <c r="K3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="L3">
         <v>0</v>
       </c>
       <c r="U3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -1064,7 +1064,7 @@
         <v>0</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C4" t="s">
         <v>4</v>
@@ -1080,7 +1080,7 @@
         <v>134</v>
       </c>
       <c r="G4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H4">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -1099,7 +1099,7 @@
         <v>0</v>
       </c>
       <c r="U4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -1107,7 +1107,7 @@
         <v>0</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C5" t="s">
         <v>3</v>
@@ -1123,7 +1123,7 @@
         <v>82</v>
       </c>
       <c r="G5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H5">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -1136,13 +1136,13 @@
         <v>8</v>
       </c>
       <c r="K5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="L5">
         <v>0</v>
       </c>
       <c r="U5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -1150,7 +1150,7 @@
         <v>0</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C6" t="s">
         <v>3</v>
@@ -1166,7 +1166,7 @@
         <v>82</v>
       </c>
       <c r="G6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H6">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -1179,13 +1179,13 @@
         <v>8</v>
       </c>
       <c r="K6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="L6">
         <v>0</v>
       </c>
       <c r="U6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -1193,7 +1193,7 @@
         <v>0</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C7" t="s">
         <v>3</v>
@@ -1209,7 +1209,7 @@
         <v>82</v>
       </c>
       <c r="G7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H7">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -1222,13 +1222,13 @@
         <v>8</v>
       </c>
       <c r="K7" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="L7">
         <v>0</v>
       </c>
       <c r="U7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -1236,7 +1236,7 @@
         <v>0</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C8" t="s">
         <v>3</v>
@@ -1252,7 +1252,7 @@
         <v>82</v>
       </c>
       <c r="G8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H8">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -1271,7 +1271,7 @@
         <v>0</v>
       </c>
       <c r="U8" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -1279,7 +1279,7 @@
         <v>0</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C9" t="s">
         <v>3</v>
@@ -1295,7 +1295,7 @@
         <v>82</v>
       </c>
       <c r="G9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H9">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -1308,13 +1308,13 @@
         <v>8</v>
       </c>
       <c r="K9" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="L9">
         <v>0</v>
       </c>
       <c r="U9" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -1322,7 +1322,7 @@
         <v>0</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C10" t="s">
         <v>3</v>
@@ -1338,7 +1338,7 @@
         <v>82</v>
       </c>
       <c r="G10" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H10">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -1357,7 +1357,7 @@
         <v>0</v>
       </c>
       <c r="U10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -1365,7 +1365,7 @@
         <v>0</v>
       </c>
       <c r="B11" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C11" t="s">
         <v>3</v>
@@ -1381,7 +1381,7 @@
         <v>82</v>
       </c>
       <c r="G11" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H11">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -1394,13 +1394,13 @@
         <v>4021.08993973114</v>
       </c>
       <c r="K11" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="L11">
         <v>0</v>
       </c>
       <c r="U11" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -1408,7 +1408,7 @@
         <v>0</v>
       </c>
       <c r="B12" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C12" t="s">
         <v>3</v>
@@ -1424,7 +1424,7 @@
         <v>82</v>
       </c>
       <c r="G12" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H12">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -1437,16 +1437,16 @@
         <v>4021.08993973114</v>
       </c>
       <c r="K12" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="L12">
         <v>0</v>
       </c>
       <c r="M12" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="U12" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -1454,7 +1454,7 @@
         <v>0</v>
       </c>
       <c r="B13" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C13" t="s">
         <v>3</v>
@@ -1470,7 +1470,7 @@
         <v>82</v>
       </c>
       <c r="G13" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H13">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -1483,14 +1483,14 @@
         <v>4021.08993973114</v>
       </c>
       <c r="K13" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="L13">
         <v>0</v>
       </c>
       <c r="O13" s="2"/>
       <c r="U13" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -1498,7 +1498,7 @@
         <v>0</v>
       </c>
       <c r="B14" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C14" t="s">
         <v>3</v>
@@ -1514,7 +1514,7 @@
         <v>82</v>
       </c>
       <c r="G14" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H14">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -1527,14 +1527,14 @@
         <v>4021.08993973114</v>
       </c>
       <c r="K14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="L14">
         <v>0</v>
       </c>
       <c r="O14" s="2"/>
       <c r="U14" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -1542,7 +1542,7 @@
         <v>0</v>
       </c>
       <c r="B15" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C15" t="s">
         <v>3</v>
@@ -1558,7 +1558,7 @@
         <v>82</v>
       </c>
       <c r="G15" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H15">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -1578,7 +1578,7 @@
       </c>
       <c r="O15" s="2"/>
       <c r="U15" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -1586,7 +1586,7 @@
         <v>0</v>
       </c>
       <c r="B16" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C16" t="s">
         <v>4</v>
@@ -1602,7 +1602,7 @@
         <v>134</v>
       </c>
       <c r="G16" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H16">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -1622,7 +1622,7 @@
       </c>
       <c r="O16" s="2"/>
       <c r="U16" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -1630,7 +1630,7 @@
         <v>0</v>
       </c>
       <c r="B17" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C17" t="s">
         <v>3</v>
@@ -1646,7 +1646,7 @@
         <v>82</v>
       </c>
       <c r="G17" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H17">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -1659,14 +1659,14 @@
         <v>4021.08993973114</v>
       </c>
       <c r="K17" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="L17">
         <v>0</v>
       </c>
       <c r="O17" s="2"/>
       <c r="U17" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -1674,7 +1674,7 @@
         <v>0</v>
       </c>
       <c r="B18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C18" t="s">
         <v>3</v>
@@ -1690,7 +1690,7 @@
         <v>82</v>
       </c>
       <c r="G18" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H18">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -1710,7 +1710,7 @@
       </c>
       <c r="O18" s="2"/>
       <c r="U18" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -1718,7 +1718,7 @@
         <v>0</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>2</v>
@@ -1734,7 +1734,7 @@
         <v>693</v>
       </c>
       <c r="G19" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H19">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -1747,19 +1747,19 @@
         <v>2397.5449116507398</v>
       </c>
       <c r="K19" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="L19">
         <v>1</v>
       </c>
       <c r="M19" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O19" t="s">
         <v>23</v>
       </c>
       <c r="P19" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="U19">
         <v>1</v>
@@ -1770,7 +1770,7 @@
         <v>0</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C20" t="s">
         <v>3</v>
@@ -1786,7 +1786,7 @@
         <v>82</v>
       </c>
       <c r="G20" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H20">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -1799,14 +1799,14 @@
         <v>392</v>
       </c>
       <c r="K20" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="L20">
         <v>0</v>
       </c>
       <c r="O20" s="2"/>
       <c r="U20" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -1814,7 +1814,7 @@
         <v>0</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C21" t="s">
         <v>3</v>
@@ -1830,7 +1830,7 @@
         <v>82</v>
       </c>
       <c r="G21" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H21">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -1843,14 +1843,14 @@
         <v>392</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="L21">
         <v>0</v>
       </c>
       <c r="O21" s="2"/>
       <c r="U21" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -1858,7 +1858,7 @@
         <v>0</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C22" t="s">
         <v>3</v>
@@ -1874,7 +1874,7 @@
         <v>82</v>
       </c>
       <c r="G22" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H22">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -1887,14 +1887,14 @@
         <v>392</v>
       </c>
       <c r="K22" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="L22">
         <v>0</v>
       </c>
       <c r="O22" s="2"/>
       <c r="U22" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -1902,7 +1902,7 @@
         <v>0</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C23" t="s">
         <v>3</v>
@@ -1918,7 +1918,7 @@
         <v>82</v>
       </c>
       <c r="G23" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H23">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -1931,14 +1931,14 @@
         <v>392</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="L23">
         <v>0</v>
       </c>
       <c r="O23" s="2"/>
       <c r="U23" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -1946,7 +1946,7 @@
         <v>5</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C24" t="s">
         <v>6</v>
@@ -1962,7 +1962,7 @@
         <v>226</v>
       </c>
       <c r="G24" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H24">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -1975,19 +1975,19 @@
         <v>10573.058588388199</v>
       </c>
       <c r="K24" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="L24">
         <v>1</v>
       </c>
       <c r="M24" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O24" t="s">
         <v>24</v>
       </c>
       <c r="P24" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="U24">
         <v>1</v>
@@ -1998,7 +1998,7 @@
         <v>5</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C25" t="s">
         <v>7</v>
@@ -2014,7 +2014,7 @@
         <v>710</v>
       </c>
       <c r="G25" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H25">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -2027,19 +2027,19 @@
         <v>10502.2256566122</v>
       </c>
       <c r="K25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L25">
         <v>1</v>
       </c>
       <c r="M25" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O25" t="s">
         <v>23</v>
       </c>
       <c r="P25" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="U25">
         <v>1</v>
@@ -2050,7 +2050,7 @@
         <v>5</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C26" t="s">
         <v>7</v>
@@ -2066,7 +2066,7 @@
         <v>710</v>
       </c>
       <c r="G26" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H26">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -2079,19 +2079,19 @@
         <v>10502.2256566122</v>
       </c>
       <c r="K26" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="L26">
         <v>1</v>
       </c>
       <c r="M26" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O26" t="s">
         <v>23</v>
       </c>
       <c r="P26" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="U26">
         <v>1</v>
@@ -2102,7 +2102,7 @@
         <v>5</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C27" t="s">
         <v>7</v>
@@ -2118,7 +2118,7 @@
         <v>710</v>
       </c>
       <c r="G27" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H27">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -2131,19 +2131,19 @@
         <v>10502.2256566122</v>
       </c>
       <c r="K27" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="L27">
         <v>1</v>
       </c>
       <c r="M27" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O27" t="s">
         <v>23</v>
       </c>
       <c r="P27" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="U27">
         <v>1</v>
@@ -2154,7 +2154,7 @@
         <v>5</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C28" t="s">
         <v>7</v>
@@ -2170,7 +2170,7 @@
         <v>710</v>
       </c>
       <c r="G28" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H28">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -2183,19 +2183,19 @@
         <v>10502.2256566122</v>
       </c>
       <c r="K28" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="L28">
         <v>1</v>
       </c>
       <c r="M28" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O28" t="s">
         <v>23</v>
       </c>
       <c r="P28" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="U28">
         <v>1</v>
@@ -2206,7 +2206,7 @@
         <v>5</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C29" t="s">
         <v>3</v>
@@ -2222,7 +2222,7 @@
         <v>82</v>
       </c>
       <c r="G29" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H29">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -2235,13 +2235,13 @@
         <v>392</v>
       </c>
       <c r="K29" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="L29">
         <v>0</v>
       </c>
       <c r="U29" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -2249,7 +2249,7 @@
         <v>5</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C30" t="s">
         <v>7</v>
@@ -2265,7 +2265,7 @@
         <v>710</v>
       </c>
       <c r="G30" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H30">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -2278,19 +2278,19 @@
         <v>10502.2256566122</v>
       </c>
       <c r="K30" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="L30">
         <v>1</v>
       </c>
       <c r="M30" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O30" t="s">
         <v>23</v>
       </c>
       <c r="P30" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="U30">
         <v>1</v>
@@ -2301,7 +2301,7 @@
         <v>5</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C31" t="s">
         <v>8</v>
@@ -2317,7 +2317,7 @@
         <v>3634</v>
       </c>
       <c r="G31" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H31">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -2330,25 +2330,25 @@
         <v>10587.095308854299</v>
       </c>
       <c r="K31" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L31">
         <v>1</v>
       </c>
       <c r="M31" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O31" t="s">
         <v>25</v>
       </c>
       <c r="P31" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="R31" t="s">
         <v>26</v>
       </c>
       <c r="S31" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="U31">
         <v>1</v>
@@ -2359,7 +2359,7 @@
         <v>5</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C32" t="s">
         <v>8</v>
@@ -2375,7 +2375,7 @@
         <v>3634</v>
       </c>
       <c r="G32" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H32">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -2388,25 +2388,25 @@
         <v>10587.095308854299</v>
       </c>
       <c r="K32" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="L32">
         <v>1</v>
       </c>
       <c r="M32" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O32" t="s">
         <v>25</v>
       </c>
       <c r="P32" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="R32" t="s">
         <v>26</v>
       </c>
       <c r="S32" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="U32">
         <v>1</v>
@@ -2417,7 +2417,7 @@
         <v>5</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C33" t="s">
         <v>8</v>
@@ -2433,7 +2433,7 @@
         <v>3634</v>
       </c>
       <c r="G33" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H33">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -2446,25 +2446,25 @@
         <v>10587.095308854299</v>
       </c>
       <c r="K33" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="L33">
         <v>1</v>
       </c>
       <c r="M33" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O33" t="s">
         <v>25</v>
       </c>
       <c r="P33" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="R33" t="s">
         <v>26</v>
       </c>
       <c r="S33" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="U33">
         <v>1</v>
@@ -2475,7 +2475,7 @@
         <v>5</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C34" t="s">
         <v>8</v>
@@ -2491,7 +2491,7 @@
         <v>3634</v>
       </c>
       <c r="G34" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H34">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -2504,25 +2504,25 @@
         <v>10587.095308854299</v>
       </c>
       <c r="K34" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="L34">
         <v>1</v>
       </c>
       <c r="M34" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O34" t="s">
         <v>25</v>
       </c>
       <c r="P34" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="R34" t="s">
         <v>26</v>
       </c>
       <c r="S34" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="U34">
         <v>1</v>
@@ -2533,7 +2533,7 @@
         <v>9</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C35" t="s">
         <v>17</v>
@@ -2549,7 +2549,7 @@
         <v>135</v>
       </c>
       <c r="G35" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H35">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -2562,19 +2562,19 @@
         <v>10105.6821775892</v>
       </c>
       <c r="K35" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="L35">
         <v>1</v>
       </c>
       <c r="M35" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O35" t="s">
         <v>27</v>
       </c>
       <c r="P35" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="U35">
         <v>1</v>
@@ -2585,7 +2585,7 @@
         <v>9</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C36" t="s">
         <v>4</v>
@@ -2601,7 +2601,7 @@
         <v>134</v>
       </c>
       <c r="G36" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H36">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -2614,13 +2614,13 @@
         <v>16</v>
       </c>
       <c r="K36" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="L36">
         <v>0</v>
       </c>
       <c r="U36" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -2628,7 +2628,7 @@
         <v>18</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C37" t="s">
         <v>3</v>
@@ -2644,7 +2644,7 @@
         <v>82</v>
       </c>
       <c r="G37" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H37">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -2657,13 +2657,13 @@
         <v>19</v>
       </c>
       <c r="K37" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="L37">
         <v>0</v>
       </c>
       <c r="U37" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -2671,7 +2671,7 @@
         <v>18</v>
       </c>
       <c r="B38" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C38" t="s">
         <v>4</v>
@@ -2687,7 +2687,7 @@
         <v>134</v>
       </c>
       <c r="G38" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H38">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -2700,13 +2700,13 @@
         <v>10066.782820697101</v>
       </c>
       <c r="K38" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="L38">
         <v>0</v>
       </c>
       <c r="U38" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="39" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -2714,7 +2714,7 @@
         <v>9</v>
       </c>
       <c r="B39" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C39" t="s">
         <v>3</v>
@@ -2730,7 +2730,7 @@
         <v>82</v>
       </c>
       <c r="G39" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H39">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -2743,13 +2743,13 @@
         <v>12910.7387536311</v>
       </c>
       <c r="K39" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="L39">
         <v>0</v>
       </c>
       <c r="U39" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -2757,7 +2757,7 @@
         <v>9</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C40" t="s">
         <v>2</v>
@@ -2773,7 +2773,7 @@
         <v>693</v>
       </c>
       <c r="G40" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H40">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -2786,19 +2786,19 @@
         <v>10066.782820697101</v>
       </c>
       <c r="K40" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L40">
         <v>1</v>
       </c>
       <c r="M40" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O40" t="s">
         <v>23</v>
       </c>
       <c r="P40" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="U40">
         <v>1</v>
@@ -2809,7 +2809,7 @@
         <v>9</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C41" t="s">
         <v>2</v>
@@ -2825,7 +2825,7 @@
         <v>693</v>
       </c>
       <c r="G41" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H41">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -2838,19 +2838,19 @@
         <v>10066.782820697101</v>
       </c>
       <c r="K41" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="L41">
         <v>1</v>
       </c>
       <c r="M41" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O41" t="s">
         <v>23</v>
       </c>
       <c r="P41" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="U41">
         <v>1</v>
@@ -2861,7 +2861,7 @@
         <v>10</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C42" t="s">
         <v>13</v>
@@ -2877,7 +2877,7 @@
         <v>22</v>
       </c>
       <c r="G42" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H42">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -2890,13 +2890,13 @@
         <v>135</v>
       </c>
       <c r="K42" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="L42">
         <v>0</v>
       </c>
       <c r="U42" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -2904,7 +2904,7 @@
         <v>10</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C43" t="s">
         <v>4</v>
@@ -2920,7 +2920,7 @@
         <v>134</v>
       </c>
       <c r="G43" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H43">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -2933,13 +2933,13 @@
         <v>12</v>
       </c>
       <c r="K43" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="L43">
         <v>0</v>
       </c>
       <c r="U43" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -2947,7 +2947,7 @@
         <v>10</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C44" t="s">
         <v>4</v>
@@ -2963,7 +2963,7 @@
         <v>134</v>
       </c>
       <c r="G44" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H44">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -2976,13 +2976,13 @@
         <v>12</v>
       </c>
       <c r="K44" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="L44">
         <v>0</v>
       </c>
       <c r="U44" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -2990,7 +2990,7 @@
         <v>19</v>
       </c>
       <c r="B45" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C45" t="s">
         <v>4</v>
@@ -3006,7 +3006,7 @@
         <v>134</v>
       </c>
       <c r="G45" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H45">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -3019,13 +3019,13 @@
         <v>8405.8620618061104</v>
       </c>
       <c r="K45" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="L45">
         <v>0</v>
       </c>
       <c r="U45" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -3033,7 +3033,7 @@
         <v>19</v>
       </c>
       <c r="B46" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C46" t="s">
         <v>4</v>
@@ -3049,7 +3049,7 @@
         <v>134</v>
       </c>
       <c r="G46" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H46">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -3062,13 +3062,13 @@
         <v>8405.8620618061104</v>
       </c>
       <c r="K46" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="L46">
         <v>0</v>
       </c>
       <c r="U46" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -3076,7 +3076,7 @@
         <v>10</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C47" t="s">
         <v>11</v>
@@ -3092,7 +3092,7 @@
         <v>1300</v>
       </c>
       <c r="G47" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H47">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -3105,19 +3105,19 @@
         <v>8405.8620618061104</v>
       </c>
       <c r="K47" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L47">
         <v>1</v>
       </c>
       <c r="M47" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O47" t="s">
         <v>23</v>
       </c>
       <c r="P47" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="U47">
         <v>1</v>
@@ -3128,7 +3128,7 @@
         <v>10</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C48" t="s">
         <v>11</v>
@@ -3144,7 +3144,7 @@
         <v>1300</v>
       </c>
       <c r="G48" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H48">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -3157,19 +3157,19 @@
         <v>8405.8620618061104</v>
       </c>
       <c r="K48" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="L48">
         <v>1</v>
       </c>
       <c r="M48" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O48" t="s">
         <v>23</v>
       </c>
       <c r="P48" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="U48">
         <v>1</v>
@@ -3180,7 +3180,7 @@
         <v>10</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C49" t="s">
         <v>11</v>
@@ -3196,7 +3196,7 @@
         <v>1300</v>
       </c>
       <c r="G49" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H49">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -3209,19 +3209,19 @@
         <v>8405.8620618061104</v>
       </c>
       <c r="K49" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="L49">
         <v>1</v>
       </c>
       <c r="M49" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O49" t="s">
         <v>23</v>
       </c>
       <c r="P49" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="U49">
         <v>1</v>
@@ -3232,7 +3232,7 @@
         <v>19</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C50" t="s">
         <v>11</v>
@@ -3248,7 +3248,7 @@
         <v>1300</v>
       </c>
       <c r="G50" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H50">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -3261,19 +3261,19 @@
         <v>8405.8620618061104</v>
       </c>
       <c r="K50" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="L50">
         <v>1</v>
       </c>
       <c r="M50" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O50" t="s">
         <v>27</v>
       </c>
       <c r="P50" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="U50">
         <v>1</v>
@@ -3284,7 +3284,7 @@
         <v>19</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C51" t="s">
         <v>12</v>
@@ -3300,7 +3300,7 @@
         <v>137</v>
       </c>
       <c r="G51" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H51">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -3313,13 +3313,13 @@
         <v>15</v>
       </c>
       <c r="K51" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="L51">
         <v>0</v>
       </c>
       <c r="U51" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -3327,7 +3327,7 @@
         <v>19</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C52" t="s">
         <v>12</v>
@@ -3343,7 +3343,7 @@
         <v>137</v>
       </c>
       <c r="G52" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H52">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -3356,13 +3356,13 @@
         <v>15</v>
       </c>
       <c r="K52" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="L52">
         <v>0</v>
       </c>
       <c r="U52" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="53" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -3370,7 +3370,7 @@
         <v>10</v>
       </c>
       <c r="B53" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C53" t="s">
         <v>12</v>
@@ -3386,7 +3386,7 @@
         <v>137</v>
       </c>
       <c r="G53" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H53">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -3399,13 +3399,13 @@
         <v>9282.1355081583297</v>
       </c>
       <c r="K53" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="L53">
         <v>0</v>
       </c>
       <c r="U53" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -3413,7 +3413,7 @@
         <v>10</v>
       </c>
       <c r="B54" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C54" t="s">
         <v>12</v>
@@ -3429,7 +3429,7 @@
         <v>137</v>
       </c>
       <c r="G54" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H54">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -3442,13 +3442,13 @@
         <v>9282.1355081583297</v>
       </c>
       <c r="K54" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="L54">
         <v>0</v>
       </c>
       <c r="U54" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="55" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -3456,7 +3456,7 @@
         <v>14</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C55" t="s">
         <v>15</v>
@@ -3472,7 +3472,7 @@
         <v>86</v>
       </c>
       <c r="G55" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H55">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -3485,19 +3485,19 @@
         <v>10744.977206715501</v>
       </c>
       <c r="K55" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="L55">
         <v>1</v>
       </c>
       <c r="M55" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O55" t="s">
         <v>30</v>
       </c>
       <c r="P55" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="U55">
         <v>1</v>
@@ -3508,7 +3508,7 @@
         <v>20</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C56" t="s">
         <v>7</v>
@@ -3524,7 +3524,7 @@
         <v>710</v>
       </c>
       <c r="G56" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H56">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -3537,13 +3537,13 @@
         <v>17</v>
       </c>
       <c r="K56" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="L56">
         <v>0</v>
       </c>
       <c r="U56" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -3551,7 +3551,7 @@
         <v>14</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C57" t="s">
         <v>7</v>
@@ -3567,7 +3567,7 @@
         <v>710</v>
       </c>
       <c r="G57" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H57">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -3580,13 +3580,13 @@
         <v>407</v>
       </c>
       <c r="K57" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="L57">
         <v>0</v>
       </c>
       <c r="U57" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -3594,7 +3594,7 @@
         <v>14</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C58" t="s">
         <v>4</v>
@@ -3610,7 +3610,7 @@
         <v>134</v>
       </c>
       <c r="G58" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H58">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -3623,13 +3623,13 @@
         <v>16</v>
       </c>
       <c r="K58" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="L58">
         <v>0</v>
       </c>
       <c r="U58" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -3637,7 +3637,7 @@
         <v>20</v>
       </c>
       <c r="B59" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C59" t="s">
         <v>7</v>
@@ -3653,7 +3653,7 @@
         <v>710</v>
       </c>
       <c r="G59" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H59">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -3666,22 +3666,22 @@
         <v>10718.466607534499</v>
       </c>
       <c r="K59" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="L59">
         <v>0</v>
       </c>
       <c r="M59" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="O59" t="s">
         <v>23</v>
       </c>
       <c r="P59" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="U59" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -3689,7 +3689,7 @@
         <v>20</v>
       </c>
       <c r="B60" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C60" t="s">
         <v>4</v>
@@ -3705,7 +3705,7 @@
         <v>134</v>
       </c>
       <c r="G60" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H60">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -3718,13 +3718,13 @@
         <v>10713.039198783999</v>
       </c>
       <c r="K60" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="L60">
         <v>0</v>
       </c>
       <c r="U60" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -3732,7 +3732,7 @@
         <v>20</v>
       </c>
       <c r="B61" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C61" t="s">
         <v>3</v>
@@ -3748,7 +3748,7 @@
         <v>82</v>
       </c>
       <c r="G61" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H61">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -3761,13 +3761,13 @@
         <v>11633.4375624042</v>
       </c>
       <c r="K61" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="L61">
         <v>0</v>
       </c>
       <c r="U61" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -3775,7 +3775,7 @@
         <v>20</v>
       </c>
       <c r="B62" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C62" t="s">
         <v>7</v>
@@ -3791,7 +3791,7 @@
         <v>710</v>
       </c>
       <c r="G62" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H62">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -3810,16 +3810,16 @@
         <v>0</v>
       </c>
       <c r="M62" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="O62" t="s">
         <v>23</v>
       </c>
       <c r="P62" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="U62" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -3827,7 +3827,7 @@
         <v>14</v>
       </c>
       <c r="B63" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C63" t="s">
         <v>7</v>
@@ -3843,7 +3843,7 @@
         <v>710</v>
       </c>
       <c r="G63" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H63">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -3856,22 +3856,22 @@
         <v>10718.466607534499</v>
       </c>
       <c r="K63" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="L63">
         <v>0</v>
       </c>
       <c r="M63" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="O63" t="s">
         <v>23</v>
       </c>
       <c r="P63" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="U63" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="64" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -3879,7 +3879,7 @@
         <v>14</v>
       </c>
       <c r="B64" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C64" t="s">
         <v>16</v>
@@ -3895,7 +3895,7 @@
         <v>62</v>
       </c>
       <c r="G64" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H64">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -3908,28 +3908,28 @@
         <v>11628.0101536537</v>
       </c>
       <c r="K64" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="L64">
         <v>0</v>
       </c>
       <c r="M64" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="O64" t="s">
         <v>28</v>
       </c>
       <c r="P64" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="R64" t="s">
         <v>29</v>
       </c>
       <c r="S64" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="U64" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="65" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -3937,7 +3937,7 @@
         <v>20</v>
       </c>
       <c r="B65" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C65" t="s">
         <v>7</v>
@@ -3953,7 +3953,7 @@
         <v>710</v>
       </c>
       <c r="G65" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H65">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -3966,13 +3966,13 @@
         <v>10718.466607534499</v>
       </c>
       <c r="K65" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="L65">
         <v>0</v>
       </c>
       <c r="U65" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="66" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -3980,7 +3980,7 @@
         <v>14</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C66" t="s">
         <v>3</v>
@@ -3996,7 +3996,7 @@
         <v>82</v>
       </c>
       <c r="G66" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H66">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -4009,13 +4009,13 @@
         <v>428</v>
       </c>
       <c r="K66" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="L66">
         <v>0</v>
       </c>
       <c r="U66" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="67" spans="1:21" x14ac:dyDescent="0.55000000000000004">
@@ -4023,7 +4023,7 @@
         <v>14</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C67" t="s">
         <v>16</v>
@@ -4039,7 +4039,7 @@
         <v>62</v>
       </c>
       <c r="G67" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H67">
         <f>ABS(分析結果[[#This Row],[after_change]]-分析結果[[#This Row],[before_change]])</f>
@@ -4052,13 +4052,13 @@
         <v>454</v>
       </c>
       <c r="K67" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="L67">
         <v>0</v>
       </c>
       <c r="U67" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.55000000000000004">

</xml_diff>